<commit_message>
[30/09] Prime Day largo: A+B+C aprovados pelo LEO (59 SKUs), P4080 e P3050 voltam; linha SP: SP-FF e SP-T podem entrar, SP-01 fora (politica), SP-PP fora (margem)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012rBhhYMg4csfyvEFcZnaje
</commit_message>
<xml_diff>
--- a/dados/PROPOSTA_PrimeDay_desconto_evento_catalogo.xlsx
+++ b/dados/PROPOSTA_PrimeDay_desconto_evento_catalogo.xlsx
@@ -2006,36 +2006,36 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>L2440-AML</t>
+          <t>SP-T</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>B0H4RY2L65</t>
+          <t>B0H3MGC36H</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Pequenos</t>
+          <t>Medios</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>228.04</v>
+        <v>462.37</v>
       </c>
       <c r="E36" t="n">
-        <v>205.24</v>
+        <v>416.13</v>
       </c>
       <c r="F36" t="n">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="G36" t="n">
-        <v>12.5</v>
+        <v>12.6</v>
       </c>
       <c r="H36" t="n">
-        <v>10.4</v>
+        <v>10.5</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -2044,40 +2044,40 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>sem tráfego recente; custo só se vender; selo pode gerar 1ª visita · ⚠️ margem no piso: pedido de 3+ empilha promo de quantidade → 12.5%</t>
+          <t>anunciado normalmente na Manual Bituqueiras (sem suspensão); margem no piso (15,7%): pedido de 3+ → 12,5%. Entrar é decisão do LEO</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>L2460-A</t>
+          <t>L2440-AML</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>B0H6QYTSNV</t>
+          <t>B0H4RY2L65</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Medios</t>
+          <t>Pequenos</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>272.57</v>
+        <v>228.04</v>
       </c>
       <c r="E37" t="n">
-        <v>245.31</v>
+        <v>205.24</v>
       </c>
       <c r="F37" t="n">
-        <v>17.3</v>
+        <v>15.8</v>
       </c>
       <c r="G37" t="n">
-        <v>14.2</v>
+        <v>12.5</v>
       </c>
       <c r="H37" t="n">
-        <v>12.1</v>
+        <v>10.4</v>
       </c>
       <c r="I37" t="n">
         <v>0</v>
@@ -2089,19 +2089,19 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>sem tráfego recente; custo só se vender; selo pode gerar 1ª visita</t>
+          <t>sem tráfego recente; custo só se vender; selo pode gerar 1ª visita · ⚠️ margem no piso: pedido de 3+ empilha promo de quantidade → 12.5%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>L2470-AML</t>
+          <t>L2460-A</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>B0H6NCDJ5C</t>
+          <t>B0H6QYTSNV</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2110,19 +2110,19 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>408.32</v>
+        <v>272.57</v>
       </c>
       <c r="E38" t="n">
-        <v>367.49</v>
+        <v>245.31</v>
       </c>
       <c r="F38" t="n">
-        <v>17.8</v>
+        <v>17.3</v>
       </c>
       <c r="G38" t="n">
-        <v>14.7</v>
+        <v>14.2</v>
       </c>
       <c r="H38" t="n">
-        <v>12.7</v>
+        <v>12.1</v>
       </c>
       <c r="I38" t="n">
         <v>0</v>
@@ -2141,12 +2141,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>L3040-A</t>
+          <t>L2470-AML</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>B0H5MJTHK2</t>
+          <t>B0H6NCDJ5C</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2155,19 +2155,19 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>296.92</v>
+        <v>408.32</v>
       </c>
       <c r="E39" t="n">
-        <v>267.23</v>
+        <v>367.49</v>
       </c>
       <c r="F39" t="n">
-        <v>16.6</v>
+        <v>17.8</v>
       </c>
       <c r="G39" t="n">
-        <v>13.4</v>
+        <v>14.7</v>
       </c>
       <c r="H39" t="n">
-        <v>11.3</v>
+        <v>12.7</v>
       </c>
       <c r="I39" t="n">
         <v>0</v>
@@ -2186,12 +2186,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>L3050-A</t>
+          <t>L3040-A</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>B0H6R85LBZ</t>
+          <t>B0H5MJTHK2</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2200,19 +2200,19 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>369.74</v>
+        <v>296.92</v>
       </c>
       <c r="E40" t="n">
-        <v>332.77</v>
+        <v>267.23</v>
       </c>
       <c r="F40" t="n">
-        <v>17.1</v>
+        <v>16.6</v>
       </c>
       <c r="G40" t="n">
-        <v>14</v>
+        <v>13.4</v>
       </c>
       <c r="H40" t="n">
-        <v>11.9</v>
+        <v>11.3</v>
       </c>
       <c r="I40" t="n">
         <v>0</v>
@@ -2231,12 +2231,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>L3060-A</t>
+          <t>L3050-A</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>B0H6R5SYVL</t>
+          <t>B0H6R85LBZ</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2245,19 +2245,19 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>396.88</v>
+        <v>369.74</v>
       </c>
       <c r="E41" t="n">
-        <v>357.19</v>
+        <v>332.77</v>
       </c>
       <c r="F41" t="n">
-        <v>16.8</v>
+        <v>17.1</v>
       </c>
       <c r="G41" t="n">
-        <v>13.7</v>
+        <v>14</v>
       </c>
       <c r="H41" t="n">
-        <v>11.6</v>
+        <v>11.9</v>
       </c>
       <c r="I41" t="n">
         <v>0</v>
@@ -2276,12 +2276,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>L3060-AML</t>
+          <t>L3060-A</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>B0H6NFGH2Q</t>
+          <t>B0H6R5SYVL</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2290,19 +2290,19 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>446.71</v>
+        <v>396.88</v>
       </c>
       <c r="E42" t="n">
-        <v>402.04</v>
+        <v>357.19</v>
       </c>
       <c r="F42" t="n">
-        <v>16.3</v>
+        <v>16.8</v>
       </c>
       <c r="G42" t="n">
-        <v>13.1</v>
+        <v>13.7</v>
       </c>
       <c r="H42" t="n">
-        <v>11</v>
+        <v>11.6</v>
       </c>
       <c r="I42" t="n">
         <v>0</v>
@@ -2321,12 +2321,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>L3060-B</t>
+          <t>L3060-AML</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>B0H6KK21H1</t>
+          <t>B0H6NFGH2Q</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2335,19 +2335,19 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>439.24</v>
+        <v>446.71</v>
       </c>
       <c r="E43" t="n">
-        <v>395.32</v>
+        <v>402.04</v>
       </c>
       <c r="F43" t="n">
-        <v>18.5</v>
+        <v>16.3</v>
       </c>
       <c r="G43" t="n">
-        <v>15.4</v>
+        <v>13.1</v>
       </c>
       <c r="H43" t="n">
-        <v>13.4</v>
+        <v>11</v>
       </c>
       <c r="I43" t="n">
         <v>0</v>
@@ -2366,12 +2366,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>L4050-A</t>
+          <t>L3060-B</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>B0H6R5XK94</t>
+          <t>B0H6KK21H1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2380,19 +2380,19 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>571.15</v>
+        <v>439.24</v>
       </c>
       <c r="E44" t="n">
-        <v>514.03</v>
+        <v>395.32</v>
       </c>
       <c r="F44" t="n">
-        <v>18.6</v>
+        <v>18.5</v>
       </c>
       <c r="G44" t="n">
-        <v>15.5</v>
+        <v>15.4</v>
       </c>
       <c r="H44" t="n">
-        <v>13.5</v>
+        <v>13.4</v>
       </c>
       <c r="I44" t="n">
         <v>0</v>
@@ -2411,12 +2411,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>L4050-B</t>
+          <t>L4050-A</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>B0H6GXK1SH</t>
+          <t>B0H6R5XK94</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2425,19 +2425,19 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>650.63</v>
+        <v>571.15</v>
       </c>
       <c r="E45" t="n">
-        <v>585.5700000000001</v>
+        <v>514.03</v>
       </c>
       <c r="F45" t="n">
-        <v>17.4</v>
+        <v>18.6</v>
       </c>
       <c r="G45" t="n">
-        <v>14.2</v>
+        <v>15.5</v>
       </c>
       <c r="H45" t="n">
-        <v>12.2</v>
+        <v>13.5</v>
       </c>
       <c r="I45" t="n">
         <v>0</v>
@@ -2456,12 +2456,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>P3040</t>
+          <t>L4050-B</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>B0H7LFY3JP</t>
+          <t>B0H6GXK1SH</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2470,19 +2470,19 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>380.01</v>
+        <v>650.63</v>
       </c>
       <c r="E46" t="n">
-        <v>342.01</v>
+        <v>585.5700000000001</v>
       </c>
       <c r="F46" t="n">
-        <v>17.3</v>
+        <v>17.4</v>
       </c>
       <c r="G46" t="n">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="H46" t="n">
-        <v>12.1</v>
+        <v>12.2</v>
       </c>
       <c r="I46" t="n">
         <v>0</v>
@@ -2501,12 +2501,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>P4050</t>
+          <t>P3040</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>B0H5MWNDKW</t>
+          <t>B0H7LFY3JP</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2515,19 +2515,19 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>701.76</v>
+        <v>380.01</v>
       </c>
       <c r="E47" t="n">
-        <v>631.58</v>
+        <v>342.01</v>
       </c>
       <c r="F47" t="n">
-        <v>16.7</v>
+        <v>17.3</v>
       </c>
       <c r="G47" t="n">
-        <v>13.5</v>
+        <v>14.1</v>
       </c>
       <c r="H47" t="n">
-        <v>11.4</v>
+        <v>12.1</v>
       </c>
       <c r="I47" t="n">
         <v>0</v>
@@ -2546,12 +2546,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>P4060</t>
+          <t>P4050</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>B0H7KTWPXB</t>
+          <t>B0H5MWNDKW</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2560,19 +2560,19 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>811.9400000000001</v>
+        <v>701.76</v>
       </c>
       <c r="E48" t="n">
-        <v>730.75</v>
+        <v>631.58</v>
       </c>
       <c r="F48" t="n">
-        <v>20</v>
+        <v>16.7</v>
       </c>
       <c r="G48" t="n">
-        <v>16.9</v>
+        <v>13.5</v>
       </c>
       <c r="H48" t="n">
-        <v>15</v>
+        <v>11.4</v>
       </c>
       <c r="I48" t="n">
         <v>0</v>
@@ -2591,12 +2591,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>P4060ALC</t>
+          <t>P4060</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>B0H6H25KJX</t>
+          <t>B0H7KTWPXB</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2605,19 +2605,19 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>988.28</v>
+        <v>811.9400000000001</v>
       </c>
       <c r="E49" t="n">
-        <v>889.45</v>
+        <v>730.75</v>
       </c>
       <c r="F49" t="n">
-        <v>17.3</v>
+        <v>20</v>
       </c>
       <c r="G49" t="n">
-        <v>14.1</v>
+        <v>16.9</v>
       </c>
       <c r="H49" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
@@ -2636,12 +2636,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PG3070</t>
+          <t>P4060ALC</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>B0H4S6J82Z</t>
+          <t>B0H6H25KJX</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2650,19 +2650,19 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>451.17</v>
+        <v>988.28</v>
       </c>
       <c r="E50" t="n">
-        <v>406.05</v>
+        <v>889.45</v>
       </c>
       <c r="F50" t="n">
-        <v>17.6</v>
+        <v>17.3</v>
       </c>
       <c r="G50" t="n">
-        <v>14.4</v>
+        <v>14.1</v>
       </c>
       <c r="H50" t="n">
-        <v>12.4</v>
+        <v>12</v>
       </c>
       <c r="I50" t="n">
         <v>0</v>
@@ -2681,12 +2681,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SP-FF</t>
+          <t>PG3070</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>B0H5X821QS</t>
+          <t>B0H4S6J82Z</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2695,19 +2695,19 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>457.17</v>
+        <v>451.17</v>
       </c>
       <c r="E51" t="n">
-        <v>411.45</v>
+        <v>406.05</v>
       </c>
       <c r="F51" t="n">
-        <v>17.5</v>
+        <v>17.6</v>
       </c>
       <c r="G51" t="n">
-        <v>14.3</v>
+        <v>14.4</v>
       </c>
       <c r="H51" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
@@ -2726,33 +2726,33 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>L4075-B</t>
+          <t>SP-FF</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>B0H6H2BTKC</t>
+          <t>B0H5X821QS</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Grandes</t>
+          <t>Medios</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>810.5</v>
+        <v>457.17</v>
       </c>
       <c r="E52" t="n">
-        <v>729.45</v>
+        <v>411.45</v>
       </c>
       <c r="F52" t="n">
-        <v>17.7</v>
+        <v>17.5</v>
       </c>
       <c r="G52" t="n">
-        <v>14.7</v>
+        <v>14.3</v>
       </c>
       <c r="H52" t="n">
-        <v>12.6</v>
+        <v>12.3</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
@@ -2764,19 +2764,19 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>sem tráfego recente; custo só se vender; selo pode gerar 1ª visita</t>
+          <t>sem tráfego recente; sem histórico de política — pode entrar</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>L4090-A</t>
+          <t>L4075-B</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>B0H6R1WBTM</t>
+          <t>B0H6H2BTKC</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2785,19 +2785,19 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>822.83</v>
+        <v>810.5</v>
       </c>
       <c r="E53" t="n">
-        <v>740.55</v>
+        <v>729.45</v>
       </c>
       <c r="F53" t="n">
-        <v>21.7</v>
+        <v>17.7</v>
       </c>
       <c r="G53" t="n">
-        <v>18.8</v>
+        <v>14.7</v>
       </c>
       <c r="H53" t="n">
-        <v>17</v>
+        <v>12.6</v>
       </c>
       <c r="I53" t="n">
         <v>0</v>
@@ -2816,12 +2816,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>L4090-B</t>
+          <t>L4090-A</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>B0H6GQB9S3</t>
+          <t>B0H6R1WBTM</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2830,19 +2830,19 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>895.15</v>
+        <v>822.83</v>
       </c>
       <c r="E54" t="n">
-        <v>805.63</v>
+        <v>740.55</v>
       </c>
       <c r="F54" t="n">
-        <v>18.4</v>
+        <v>21.7</v>
       </c>
       <c r="G54" t="n">
-        <v>15.4</v>
+        <v>18.8</v>
       </c>
       <c r="H54" t="n">
-        <v>13.4</v>
+        <v>17</v>
       </c>
       <c r="I54" t="n">
         <v>0</v>
@@ -2861,12 +2861,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>P4070RA</t>
+          <t>L4090-B</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>B0H4NGLNQ4</t>
+          <t>B0H6GQB9S3</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2875,19 +2875,19 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>1290.49</v>
+        <v>895.15</v>
       </c>
       <c r="E55" t="n">
-        <v>1161.44</v>
+        <v>805.63</v>
       </c>
       <c r="F55" t="n">
-        <v>16.9</v>
+        <v>18.4</v>
       </c>
       <c r="G55" t="n">
-        <v>13.7</v>
+        <v>15.4</v>
       </c>
       <c r="H55" t="n">
-        <v>11.7</v>
+        <v>13.4</v>
       </c>
       <c r="I55" t="n">
         <v>0</v>
@@ -2906,12 +2906,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>P4075</t>
+          <t>P4070RA</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>B0H7KZNQ9G</t>
+          <t>B0H4NGLNQ4</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2920,19 +2920,19 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>923.64</v>
+        <v>1290.49</v>
       </c>
       <c r="E56" t="n">
-        <v>831.28</v>
+        <v>1161.44</v>
       </c>
       <c r="F56" t="n">
-        <v>19.1</v>
+        <v>16.9</v>
       </c>
       <c r="G56" t="n">
-        <v>16.1</v>
+        <v>13.7</v>
       </c>
       <c r="H56" t="n">
-        <v>14.1</v>
+        <v>11.7</v>
       </c>
       <c r="I56" t="n">
         <v>0</v>
@@ -2951,12 +2951,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>P4075ALC</t>
+          <t>P4075</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>B0H72BV1KC</t>
+          <t>B0H7KZNQ9G</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2965,19 +2965,19 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>1135.46</v>
+        <v>923.64</v>
       </c>
       <c r="E57" t="n">
-        <v>1021.91</v>
+        <v>831.28</v>
       </c>
       <c r="F57" t="n">
-        <v>17.6</v>
+        <v>19.1</v>
       </c>
       <c r="G57" t="n">
-        <v>14.5</v>
+        <v>16.1</v>
       </c>
       <c r="H57" t="n">
-        <v>12.5</v>
+        <v>14.1</v>
       </c>
       <c r="I57" t="n">
         <v>0</v>
@@ -2996,12 +2996,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>P4090</t>
+          <t>P4075ALC</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>B0H7KTX9Y2</t>
+          <t>B0H72BV1KC</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -3010,19 +3010,19 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1433.32</v>
+        <v>1135.46</v>
       </c>
       <c r="E58" t="n">
-        <v>1289.99</v>
+        <v>1021.91</v>
       </c>
       <c r="F58" t="n">
-        <v>17.3</v>
+        <v>17.6</v>
       </c>
       <c r="G58" t="n">
-        <v>14.1</v>
+        <v>14.5</v>
       </c>
       <c r="H58" t="n">
-        <v>12.1</v>
+        <v>12.5</v>
       </c>
       <c r="I58" t="n">
         <v>0</v>
@@ -3041,12 +3041,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>P4090ALC</t>
+          <t>P4090</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>B0H72JR46M</t>
+          <t>B0H7KTX9Y2</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3055,19 +3055,19 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1527.88</v>
+        <v>1433.32</v>
       </c>
       <c r="E59" t="n">
-        <v>1375.09</v>
+        <v>1289.99</v>
       </c>
       <c r="F59" t="n">
-        <v>16.9</v>
+        <v>17.3</v>
       </c>
       <c r="G59" t="n">
-        <v>13.7</v>
+        <v>14.1</v>
       </c>
       <c r="H59" t="n">
-        <v>11.7</v>
+        <v>12.1</v>
       </c>
       <c r="I59" t="n">
         <v>0</v>
@@ -3086,81 +3086,81 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>P3060</t>
+          <t>P4090ALC</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>B0H4NLBG1Y</t>
+          <t>B0H72JR46M</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Medios</t>
+          <t>Grandes</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>511.42</v>
+        <v>1527.88</v>
       </c>
       <c r="E60" t="n">
-        <v>460.28</v>
+        <v>1375.09</v>
       </c>
       <c r="F60" t="n">
-        <v>22.6</v>
+        <v>16.9</v>
       </c>
       <c r="G60" t="n">
-        <v>19.7</v>
+        <v>13.7</v>
       </c>
       <c r="H60" t="n">
-        <v>17.8</v>
+        <v>11.7</v>
       </c>
       <c r="I60" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>JÁ CRIADO</t>
+          <t>C — opcional</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>EC-017 / EC-019</t>
+          <t>sem tráfego recente; custo só se vender; selo pode gerar 1ª visita</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PXM</t>
+          <t>P3060</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>B0H4S3FHG6</t>
+          <t>B0H4NLBG1Y</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Pequenos</t>
+          <t>Medios</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>203.54</v>
+        <v>511.42</v>
       </c>
       <c r="E61" t="n">
-        <v>183.19</v>
+        <v>460.28</v>
       </c>
       <c r="F61" t="n">
-        <v>15</v>
+        <v>22.6</v>
       </c>
       <c r="G61" t="n">
-        <v>11.7</v>
+        <v>19.7</v>
       </c>
       <c r="H61" t="n">
-        <v>9.5</v>
+        <v>17.8</v>
       </c>
       <c r="I61" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="J61" t="inlineStr">
         <is>
@@ -3169,88 +3169,88 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>EC-017 / EC-019 · ⚠️ margem no piso: pedido de 3+ empilha promo de quantidade → 11.7%</t>
+          <t>EC-017 / EC-019</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>P3070</t>
+          <t>PXM</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>B0H63FKGPJ</t>
+          <t>B0H4S3FHG6</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Medios</t>
+          <t>Pequenos</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>616.1799999999999</v>
+        <v>203.54</v>
       </c>
       <c r="E62" t="n">
-        <v>554.5599999999999</v>
+        <v>183.19</v>
       </c>
       <c r="F62" t="n">
-        <v>20.3</v>
+        <v>15</v>
       </c>
       <c r="G62" t="n">
-        <v>17.3</v>
+        <v>11.7</v>
       </c>
       <c r="H62" t="n">
-        <v>15.3</v>
+        <v>9.5</v>
       </c>
       <c r="I62" t="n">
-        <v>86</v>
+        <v>17</v>
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>JÁ NO EVENTO</t>
+          <t>JÁ CRIADO</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Melhor Oferta inscrita — não empilha; não criar desconto</t>
+          <t>EC-017 / EC-019 · ⚠️ margem no piso: pedido de 3+ empilha promo de quantidade → 11.7%</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>PXP</t>
+          <t>P3070</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>B0H4S7ZKXS</t>
+          <t>B0H63FKGPJ</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Pequenos</t>
+          <t>Medios</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>167.89</v>
+        <v>616.1799999999999</v>
       </c>
       <c r="E63" t="n">
-        <v>151.1</v>
+        <v>554.5599999999999</v>
       </c>
       <c r="F63" t="n">
-        <v>13.4</v>
+        <v>20.3</v>
       </c>
       <c r="G63" t="n">
-        <v>10</v>
+        <v>17.3</v>
       </c>
       <c r="H63" t="n">
-        <v>7.7</v>
+        <v>15.3</v>
       </c>
       <c r="I63" t="n">
-        <v>36</v>
+        <v>86</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
@@ -3266,12 +3266,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>L2025-T</t>
+          <t>PXP</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>B0H6C5CTSC</t>
+          <t>B0H4S7ZKXS</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -3280,43 +3280,43 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>132.9</v>
+        <v>167.89</v>
       </c>
       <c r="E64" t="n">
-        <v>119.61</v>
+        <v>151.1</v>
       </c>
       <c r="F64" t="n">
-        <v>13.1</v>
+        <v>13.4</v>
       </c>
       <c r="G64" t="n">
-        <v>9.800000000000001</v>
+        <v>10</v>
       </c>
       <c r="H64" t="n">
-        <v>7.6</v>
+        <v>7.7</v>
       </c>
       <c r="I64" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>FORA</t>
+          <t>JÁ NO EVENTO</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (13.1%)</t>
+          <t>Melhor Oferta inscrita — não empilha; não criar desconto</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>L1618-T</t>
+          <t>L2025-T</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>B0H3QQLFFY</t>
+          <t>B0H6C5CTSC</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -3325,22 +3325,22 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>116</v>
+        <v>132.9</v>
       </c>
       <c r="E65" t="n">
-        <v>104.4</v>
+        <v>119.61</v>
       </c>
       <c r="F65" t="n">
-        <v>11.9</v>
+        <v>13.1</v>
       </c>
       <c r="G65" t="n">
-        <v>8.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H65" t="n">
-        <v>6.3</v>
+        <v>7.6</v>
       </c>
       <c r="I65" t="n">
-        <v>82</v>
+        <v>100</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
@@ -3349,43 +3349,43 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (11.9%)</t>
+          <t>abaixo do piso a 10% (13.1%)</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Q2460-B</t>
+          <t>L1618-T</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>B0H7YNMBBK</t>
+          <t>B0H3QQLFFY</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Medios</t>
+          <t>Pequenos</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>360.97</v>
+        <v>116</v>
       </c>
       <c r="E66" t="n">
-        <v>324.87</v>
+        <v>104.4</v>
       </c>
       <c r="F66" t="n">
-        <v>13</v>
+        <v>11.9</v>
       </c>
       <c r="G66" t="n">
-        <v>9.6</v>
+        <v>8.5</v>
       </c>
       <c r="H66" t="n">
-        <v>7.4</v>
+        <v>6.3</v>
       </c>
       <c r="I66" t="n">
-        <v>36</v>
+        <v>82</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
@@ -3394,19 +3394,19 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>13,0% a 10% (abaixo do piso) e sem preço de referência</t>
+          <t>abaixo do piso a 10% (11.9%)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>PG2460</t>
+          <t>Q2460-B</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>B0H5MDZQDG</t>
+          <t>B0H7YNMBBK</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -3415,22 +3415,22 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>248.75</v>
+        <v>360.97</v>
       </c>
       <c r="E67" t="n">
-        <v>223.88</v>
+        <v>324.87</v>
       </c>
       <c r="F67" t="n">
-        <v>16.7</v>
+        <v>13</v>
       </c>
       <c r="G67" t="n">
-        <v>13.5</v>
+        <v>9.6</v>
       </c>
       <c r="H67" t="n">
-        <v>11.5</v>
+        <v>7.4</v>
       </c>
       <c r="I67" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
@@ -3439,43 +3439,43 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>sem preço de referência — desconto invisível; recuperar referência p/ Black Friday</t>
+          <t>13,0% a 10% (abaixo do piso) e sem preço de referência</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>L1623-T</t>
+          <t>PG2460</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>B0H6C894TV</t>
+          <t>B0H5MDZQDG</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Pequenos</t>
+          <t>Medios</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>123.93</v>
+        <v>248.75</v>
       </c>
       <c r="E68" t="n">
-        <v>111.54</v>
+        <v>223.88</v>
       </c>
       <c r="F68" t="n">
-        <v>11.4</v>
+        <v>16.7</v>
       </c>
       <c r="G68" t="n">
-        <v>8</v>
+        <v>13.5</v>
       </c>
       <c r="H68" t="n">
-        <v>5.7</v>
+        <v>11.5</v>
       </c>
       <c r="I68" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
@@ -3484,19 +3484,19 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (11.4%)</t>
+          <t>sem preço de referência — desconto invisível; recuperar referência p/ Black Friday</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>L2030-B</t>
+          <t>L1623-T</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>B0H4RV67FF</t>
+          <t>B0H6C894TV</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3505,19 +3505,19 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>153.72</v>
+        <v>123.93</v>
       </c>
       <c r="E69" t="n">
-        <v>138.35</v>
+        <v>111.54</v>
       </c>
       <c r="F69" t="n">
-        <v>12.8</v>
+        <v>11.4</v>
       </c>
       <c r="G69" t="n">
-        <v>9.4</v>
+        <v>8</v>
       </c>
       <c r="H69" t="n">
-        <v>7.2</v>
+        <v>5.7</v>
       </c>
       <c r="I69" t="n">
         <v>10</v>
@@ -3529,19 +3529,19 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (12.8%)</t>
+          <t>abaixo do piso a 10% (11.4%)</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>L1618-B</t>
+          <t>L2030-B</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>B0H6KPN1XS</t>
+          <t>B0H4RV67FF</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -3550,22 +3550,22 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>129.9</v>
+        <v>153.72</v>
       </c>
       <c r="E70" t="n">
-        <v>116.91</v>
+        <v>138.35</v>
       </c>
       <c r="F70" t="n">
-        <v>13.7</v>
+        <v>12.8</v>
       </c>
       <c r="G70" t="n">
-        <v>10.4</v>
+        <v>9.4</v>
       </c>
       <c r="H70" t="n">
-        <v>8.199999999999999</v>
+        <v>7.2</v>
       </c>
       <c r="I70" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
@@ -3574,19 +3574,19 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (13.7%)</t>
+          <t>abaixo do piso a 10% (12.8%)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>L2030</t>
+          <t>L1618-B</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>B0H6CCHT65</t>
+          <t>B0H6KPN1XS</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -3595,19 +3595,19 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>119.22</v>
+        <v>129.9</v>
       </c>
       <c r="E71" t="n">
-        <v>107.3</v>
+        <v>116.91</v>
       </c>
       <c r="F71" t="n">
-        <v>12.8</v>
+        <v>13.7</v>
       </c>
       <c r="G71" t="n">
-        <v>9.4</v>
+        <v>10.4</v>
       </c>
       <c r="H71" t="n">
-        <v>7.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I71" t="n">
         <v>8</v>
@@ -3619,19 +3619,19 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (12.8%)</t>
+          <t>abaixo do piso a 10% (13.7%)</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>L2025-B</t>
+          <t>L2030</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>B0H6L3552G</t>
+          <t>B0H6CCHT65</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -3640,22 +3640,22 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>139.9</v>
+        <v>119.22</v>
       </c>
       <c r="E72" t="n">
-        <v>125.91</v>
+        <v>107.3</v>
       </c>
       <c r="F72" t="n">
-        <v>11.2</v>
+        <v>12.8</v>
       </c>
       <c r="G72" t="n">
-        <v>7.7</v>
+        <v>9.4</v>
       </c>
       <c r="H72" t="n">
-        <v>5.5</v>
+        <v>7.2</v>
       </c>
       <c r="I72" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
@@ -3664,43 +3664,43 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (11.2%)</t>
+          <t>abaixo do piso a 10% (12.8%)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Q3060-B</t>
+          <t>L2025-B</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>B0H51M7C59</t>
+          <t>B0H6L3552G</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Medios</t>
+          <t>Pequenos</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>532.9299999999999</v>
+        <v>139.9</v>
       </c>
       <c r="E73" t="n">
-        <v>479.64</v>
+        <v>125.91</v>
       </c>
       <c r="F73" t="n">
-        <v>12.6</v>
+        <v>11.2</v>
       </c>
       <c r="G73" t="n">
-        <v>9.199999999999999</v>
+        <v>7.7</v>
       </c>
       <c r="H73" t="n">
-        <v>6.9</v>
+        <v>5.5</v>
       </c>
       <c r="I73" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -3709,43 +3709,43 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (12.6%)</t>
+          <t>abaixo do piso a 10% (11.2%)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>L2030-T</t>
+          <t>Q3060-B</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>B0H77661G6</t>
+          <t>B0H51M7C59</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Pequenos</t>
+          <t>Medios</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>143.13</v>
+        <v>532.9299999999999</v>
       </c>
       <c r="E74" t="n">
-        <v>128.82</v>
+        <v>479.64</v>
       </c>
       <c r="F74" t="n">
-        <v>13</v>
+        <v>12.6</v>
       </c>
       <c r="G74" t="n">
-        <v>9.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H74" t="n">
-        <v>7.4</v>
+        <v>6.9</v>
       </c>
       <c r="I74" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
@@ -3754,19 +3754,19 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (13.0%)</t>
+          <t>abaixo do piso a 10% (12.6%)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>L2430-B</t>
+          <t>L2030-T</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>B0H6KY3BZD</t>
+          <t>B0H77661G6</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -3775,19 +3775,19 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>198.03</v>
+        <v>143.13</v>
       </c>
       <c r="E75" t="n">
-        <v>178.23</v>
+        <v>128.82</v>
       </c>
       <c r="F75" t="n">
-        <v>11.8</v>
+        <v>13</v>
       </c>
       <c r="G75" t="n">
-        <v>8.4</v>
+        <v>9.6</v>
       </c>
       <c r="H75" t="n">
-        <v>6.2</v>
+        <v>7.4</v>
       </c>
       <c r="I75" t="n">
         <v>5</v>
@@ -3799,19 +3799,19 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (11.8%)</t>
+          <t>abaixo do piso a 10% (13.0%)</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>EMB-03</t>
+          <t>L2430-B</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>B0H52SC552</t>
+          <t>B0H6KY3BZD</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -3820,22 +3820,22 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>195.21</v>
+        <v>198.03</v>
       </c>
       <c r="E76" t="n">
-        <v>175.69</v>
+        <v>178.23</v>
       </c>
       <c r="F76" t="n">
-        <v>14.3</v>
+        <v>11.8</v>
       </c>
       <c r="G76" t="n">
-        <v>11</v>
+        <v>8.4</v>
       </c>
       <c r="H76" t="n">
-        <v>8.800000000000001</v>
+        <v>6.2</v>
       </c>
       <c r="I76" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -3844,19 +3844,19 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>liquidação à parte (EC-006, decisão da Dianna)</t>
+          <t>abaixo do piso a 10% (11.8%)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Q2430-B</t>
+          <t>EMB-03</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>B0H4X43F5T</t>
+          <t>B0H52SC552</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -3865,19 +3865,19 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>273.9</v>
+        <v>195.21</v>
       </c>
       <c r="E77" t="n">
-        <v>246.51</v>
+        <v>175.69</v>
       </c>
       <c r="F77" t="n">
-        <v>11.3</v>
+        <v>14.3</v>
       </c>
       <c r="G77" t="n">
-        <v>7.8</v>
+        <v>11</v>
       </c>
       <c r="H77" t="n">
-        <v>5.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I77" t="n">
         <v>4</v>
@@ -3889,40 +3889,40 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (11.3%)</t>
+          <t>liquidação à parte (EC-006, decisão da Dianna)</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>PG3060</t>
+          <t>Q2430-B</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>B0H7T7K23P</t>
+          <t>B0H4X43F5T</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Medios</t>
+          <t>Pequenos</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>321.21</v>
+        <v>273.9</v>
       </c>
       <c r="E78" t="n">
-        <v>289.09</v>
+        <v>246.51</v>
       </c>
       <c r="F78" t="n">
-        <v>14.7</v>
+        <v>11.3</v>
       </c>
       <c r="G78" t="n">
-        <v>11.5</v>
+        <v>7.8</v>
       </c>
       <c r="H78" t="n">
-        <v>9.300000000000001</v>
+        <v>5.6</v>
       </c>
       <c r="I78" t="n">
         <v>4</v>
@@ -3934,43 +3934,43 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (14.7%)</t>
+          <t>abaixo do piso a 10% (11.3%)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>L1618-A</t>
+          <t>PG3060</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>B0H4NRG51Q</t>
+          <t>B0H7T7K23P</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Pequenos</t>
+          <t>Medios</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>104.9</v>
+        <v>321.21</v>
       </c>
       <c r="E79" t="n">
-        <v>94.41</v>
+        <v>289.09</v>
       </c>
       <c r="F79" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="G79" t="n">
         <v>11.5</v>
       </c>
-      <c r="G79" t="n">
-        <v>8.1</v>
-      </c>
       <c r="H79" t="n">
-        <v>5.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
@@ -3979,19 +3979,19 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (11.5%)</t>
+          <t>abaixo do piso a 10% (14.7%)</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>P2030</t>
+          <t>L1618-A</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>B0H51H5B4D</t>
+          <t>B0H4NRG51Q</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4000,19 +4000,19 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>219.68</v>
+        <v>104.9</v>
       </c>
       <c r="E80" t="n">
-        <v>197.71</v>
+        <v>94.41</v>
       </c>
       <c r="F80" t="n">
-        <v>14.4</v>
+        <v>11.5</v>
       </c>
       <c r="G80" t="n">
-        <v>11.1</v>
+        <v>8.1</v>
       </c>
       <c r="H80" t="n">
-        <v>8.9</v>
+        <v>5.9</v>
       </c>
       <c r="I80" t="n">
         <v>3</v>
@@ -4024,40 +4024,40 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (14.4%)</t>
+          <t>abaixo do piso a 10% (11.5%)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>PG2470</t>
+          <t>P2030</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>B0H7T71WHG</t>
+          <t>B0H51H5B4D</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Medios</t>
+          <t>Pequenos</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>360.6</v>
+        <v>219.68</v>
       </c>
       <c r="E81" t="n">
-        <v>324.54</v>
+        <v>197.71</v>
       </c>
       <c r="F81" t="n">
-        <v>14.1</v>
+        <v>14.4</v>
       </c>
       <c r="G81" t="n">
-        <v>10.8</v>
+        <v>11.1</v>
       </c>
       <c r="H81" t="n">
-        <v>8.699999999999999</v>
+        <v>8.9</v>
       </c>
       <c r="I81" t="n">
         <v>3</v>
@@ -4069,43 +4069,43 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (14.1%)</t>
+          <t>abaixo do piso a 10% (14.4%)</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>EMB-03P</t>
+          <t>PG2470</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>B0H73CH37Y</t>
+          <t>B0H7T71WHG</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Pequenos</t>
+          <t>Medios</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>245.9</v>
+        <v>360.6</v>
       </c>
       <c r="E82" t="n">
-        <v>221.31</v>
+        <v>324.54</v>
       </c>
       <c r="F82" t="n">
-        <v>13.7</v>
+        <v>14.1</v>
       </c>
       <c r="G82" t="n">
-        <v>10.4</v>
+        <v>10.8</v>
       </c>
       <c r="H82" t="n">
-        <v>8.199999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I82" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
@@ -4114,19 +4114,19 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>liquidação à parte (EC-006, decisão da Dianna)</t>
+          <t>abaixo do piso a 10% (14.1%)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>L2030-A</t>
+          <t>EMB-03P</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>B0H6XW8YF8</t>
+          <t>B0H73CH37Y</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -4135,19 +4135,19 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>141.9</v>
+        <v>245.9</v>
       </c>
       <c r="E83" t="n">
-        <v>127.71</v>
+        <v>221.31</v>
       </c>
       <c r="F83" t="n">
-        <v>12.9</v>
+        <v>13.7</v>
       </c>
       <c r="G83" t="n">
-        <v>9.5</v>
+        <v>10.4</v>
       </c>
       <c r="H83" t="n">
-        <v>7.4</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="I83" t="n">
         <v>2</v>
@@ -4159,19 +4159,19 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (12.9%)</t>
+          <t>liquidação à parte (EC-006, decisão da Dianna)</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>L2450-AML</t>
+          <t>L2030-A</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>B0H62YWD84</t>
+          <t>B0H6XW8YF8</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -4180,19 +4180,19 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>259.9</v>
+        <v>141.9</v>
       </c>
       <c r="E84" t="n">
-        <v>233.91</v>
+        <v>127.71</v>
       </c>
       <c r="F84" t="n">
-        <v>12</v>
+        <v>12.9</v>
       </c>
       <c r="G84" t="n">
-        <v>8.6</v>
+        <v>9.5</v>
       </c>
       <c r="H84" t="n">
-        <v>6.3</v>
+        <v>7.4</v>
       </c>
       <c r="I84" t="n">
         <v>2</v>
@@ -4204,19 +4204,19 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (12.0%)</t>
+          <t>abaixo do piso a 10% (12.9%)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>L2450-B</t>
+          <t>L2450-AML</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>B0H6KLWTPC</t>
+          <t>B0H62YWD84</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -4225,19 +4225,19 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>284.39</v>
+        <v>259.9</v>
       </c>
       <c r="E85" t="n">
-        <v>255.95</v>
+        <v>233.91</v>
       </c>
       <c r="F85" t="n">
-        <v>13.2</v>
+        <v>12</v>
       </c>
       <c r="G85" t="n">
-        <v>9.800000000000001</v>
+        <v>8.6</v>
       </c>
       <c r="H85" t="n">
-        <v>7.6</v>
+        <v>6.3</v>
       </c>
       <c r="I85" t="n">
         <v>2</v>
@@ -4249,19 +4249,19 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (13.2%)</t>
+          <t>abaixo do piso a 10% (12.0%)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>P2430</t>
+          <t>L2450-B</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>B0H7KWNLZ4</t>
+          <t>B0H6KLWTPC</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -4270,19 +4270,19 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>244.29</v>
+        <v>284.39</v>
       </c>
       <c r="E86" t="n">
-        <v>219.86</v>
+        <v>255.95</v>
       </c>
       <c r="F86" t="n">
-        <v>14.7</v>
+        <v>13.2</v>
       </c>
       <c r="G86" t="n">
-        <v>11.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H86" t="n">
-        <v>9.199999999999999</v>
+        <v>7.6</v>
       </c>
       <c r="I86" t="n">
         <v>2</v>
@@ -4294,19 +4294,19 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (14.7%)</t>
+          <t>abaixo do piso a 10% (13.2%)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SP-PP</t>
+          <t>P2430</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>B0H5X97DR7</t>
+          <t>B0H7KWNLZ4</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -4315,19 +4315,19 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>258.97</v>
+        <v>244.29</v>
       </c>
       <c r="E87" t="n">
-        <v>233.07</v>
+        <v>219.86</v>
       </c>
       <c r="F87" t="n">
-        <v>11.8</v>
+        <v>14.7</v>
       </c>
       <c r="G87" t="n">
-        <v>8.300000000000001</v>
+        <v>11.4</v>
       </c>
       <c r="H87" t="n">
-        <v>6.1</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I87" t="n">
         <v>2</v>
@@ -4339,40 +4339,40 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (11.8%)</t>
+          <t>abaixo do piso a 10% (14.7%)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>P3060ALC</t>
+          <t>SP-PP</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>B0H5LJ939G</t>
+          <t>B0H5X97DR7</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Medios</t>
+          <t>Pequenos</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>629.08</v>
+        <v>258.97</v>
       </c>
       <c r="E88" t="n">
-        <v>566.17</v>
+        <v>233.07</v>
       </c>
       <c r="F88" t="n">
-        <v>14.3</v>
+        <v>11.8</v>
       </c>
       <c r="G88" t="n">
-        <v>11</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H88" t="n">
-        <v>8.800000000000001</v>
+        <v>6.1</v>
       </c>
       <c r="I88" t="n">
         <v>2</v>
@@ -4384,43 +4384,43 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (14.3%)</t>
+          <t>abaixo do piso a 10% (11.8%)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>L1623</t>
+          <t>P3060ALC</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>B0H5N4TR7B</t>
+          <t>B0H5LJ939G</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Pequenos</t>
+          <t>Medios</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>109.9</v>
+        <v>629.08</v>
       </c>
       <c r="E89" t="n">
-        <v>98.91</v>
+        <v>566.17</v>
       </c>
       <c r="F89" t="n">
-        <v>13.6</v>
+        <v>14.3</v>
       </c>
       <c r="G89" t="n">
-        <v>10.3</v>
+        <v>11</v>
       </c>
       <c r="H89" t="n">
-        <v>8.1</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I89" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
@@ -4429,19 +4429,19 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (13.6%)</t>
+          <t>abaixo do piso a 10% (14.3%)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>L1623-B</t>
+          <t>L1623</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>B0H6KT72NN</t>
+          <t>B0H5N4TR7B</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -4450,19 +4450,19 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>137.9</v>
+        <v>109.9</v>
       </c>
       <c r="E90" t="n">
-        <v>124.11</v>
+        <v>98.91</v>
       </c>
       <c r="F90" t="n">
-        <v>13.1</v>
+        <v>13.6</v>
       </c>
       <c r="G90" t="n">
-        <v>9.800000000000001</v>
+        <v>10.3</v>
       </c>
       <c r="H90" t="n">
-        <v>7.6</v>
+        <v>8.1</v>
       </c>
       <c r="I90" t="n">
         <v>1</v>
@@ -4474,19 +4474,19 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (13.1%)</t>
+          <t>abaixo do piso a 10% (13.6%)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>L2025</t>
+          <t>L1623-B</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>B0H4WPPLZB</t>
+          <t>B0H6KT72NN</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -4495,19 +4495,19 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>113.11</v>
+        <v>137.9</v>
       </c>
       <c r="E91" t="n">
-        <v>101.8</v>
+        <v>124.11</v>
       </c>
       <c r="F91" t="n">
-        <v>12.9</v>
+        <v>13.1</v>
       </c>
       <c r="G91" t="n">
-        <v>9.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H91" t="n">
-        <v>7.3</v>
+        <v>7.6</v>
       </c>
       <c r="I91" t="n">
         <v>1</v>
@@ -4519,19 +4519,19 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (12.9%)</t>
+          <t>abaixo do piso a 10% (13.1%)</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>L2025-A</t>
+          <t>L2025</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>B0H6XYM5GF</t>
+          <t>B0H4WPPLZB</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -4540,19 +4540,19 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>127.9</v>
+        <v>113.11</v>
       </c>
       <c r="E92" t="n">
-        <v>115.11</v>
+        <v>101.8</v>
       </c>
       <c r="F92" t="n">
-        <v>13.1</v>
+        <v>12.9</v>
       </c>
       <c r="G92" t="n">
-        <v>9.699999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="H92" t="n">
-        <v>7.5</v>
+        <v>7.3</v>
       </c>
       <c r="I92" t="n">
         <v>1</v>
@@ -4564,19 +4564,19 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (13.1%)</t>
+          <t>abaixo do piso a 10% (12.9%)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>L2425-A</t>
+          <t>L2025-A</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>B0H6XV8Z59</t>
+          <t>B0H6XYM5GF</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -4585,19 +4585,19 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>160.08</v>
+        <v>127.9</v>
       </c>
       <c r="E93" t="n">
-        <v>144.07</v>
+        <v>115.11</v>
       </c>
       <c r="F93" t="n">
-        <v>12.6</v>
+        <v>13.1</v>
       </c>
       <c r="G93" t="n">
-        <v>9.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H93" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="I93" t="n">
         <v>1</v>
@@ -4609,19 +4609,19 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (12.6%)</t>
+          <t>abaixo do piso a 10% (13.1%)</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>L2430-A</t>
+          <t>L2425-A</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>B0H6XM9LGJ</t>
+          <t>B0H6XV8Z59</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -4630,19 +4630,19 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>178.49</v>
+        <v>160.08</v>
       </c>
       <c r="E94" t="n">
-        <v>160.64</v>
+        <v>144.07</v>
       </c>
       <c r="F94" t="n">
-        <v>12.2</v>
+        <v>12.6</v>
       </c>
       <c r="G94" t="n">
-        <v>8.800000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H94" t="n">
-        <v>6.6</v>
+        <v>7</v>
       </c>
       <c r="I94" t="n">
         <v>1</v>
@@ -4654,19 +4654,19 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (12.2%)</t>
+          <t>abaixo do piso a 10% (12.6%)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>L2440-B</t>
+          <t>L2430-A</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>B0H5M7DCH6</t>
+          <t>B0H6XM9LGJ</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -4675,19 +4675,19 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>231.66</v>
+        <v>178.49</v>
       </c>
       <c r="E95" t="n">
-        <v>208.49</v>
+        <v>160.64</v>
       </c>
       <c r="F95" t="n">
-        <v>13.2</v>
+        <v>12.2</v>
       </c>
       <c r="G95" t="n">
-        <v>9.9</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="H95" t="n">
-        <v>7.7</v>
+        <v>6.6</v>
       </c>
       <c r="I95" t="n">
         <v>1</v>
@@ -4699,19 +4699,19 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (13.2%)</t>
+          <t>abaixo do piso a 10% (12.2%)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>L2450-A</t>
+          <t>L2440-B</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>B0H6XYVBKH</t>
+          <t>B0H5M7DCH6</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -4720,19 +4720,19 @@
         </is>
       </c>
       <c r="D96" t="n">
-        <v>253.58</v>
+        <v>231.66</v>
       </c>
       <c r="E96" t="n">
-        <v>228.22</v>
+        <v>208.49</v>
       </c>
       <c r="F96" t="n">
-        <v>13.8</v>
+        <v>13.2</v>
       </c>
       <c r="G96" t="n">
-        <v>10.5</v>
+        <v>9.9</v>
       </c>
       <c r="H96" t="n">
-        <v>8.300000000000001</v>
+        <v>7.7</v>
       </c>
       <c r="I96" t="n">
         <v>1</v>
@@ -4744,19 +4744,19 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (13.8%)</t>
+          <t>abaixo do piso a 10% (13.2%)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>P2025</t>
+          <t>L2450-A</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>B0H7L6HYFW</t>
+          <t>B0H6XYVBKH</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -4765,19 +4765,19 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>198.79</v>
+        <v>253.58</v>
       </c>
       <c r="E97" t="n">
-        <v>178.91</v>
+        <v>228.22</v>
       </c>
       <c r="F97" t="n">
-        <v>14.2</v>
+        <v>13.8</v>
       </c>
       <c r="G97" t="n">
-        <v>10.9</v>
+        <v>10.5</v>
       </c>
       <c r="H97" t="n">
-        <v>8.800000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I97" t="n">
         <v>1</v>
@@ -4789,40 +4789,40 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (14.2%)</t>
+          <t>abaixo do piso a 10% (13.8%)</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>P3050ALC</t>
+          <t>P2025</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>B0H6C92MLT</t>
+          <t>B0H7L6HYFW</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Medios</t>
+          <t>Pequenos</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>623.5</v>
+        <v>198.79</v>
       </c>
       <c r="E98" t="n">
-        <v>561.15</v>
+        <v>178.91</v>
       </c>
       <c r="F98" t="n">
-        <v>14.1</v>
+        <v>14.2</v>
       </c>
       <c r="G98" t="n">
-        <v>10.8</v>
+        <v>10.9</v>
       </c>
       <c r="H98" t="n">
-        <v>8.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="I98" t="n">
         <v>1</v>
@@ -4834,19 +4834,19 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>abaixo do piso a 10% (14.1%)</t>
+          <t>abaixo do piso a 10% (14.2%)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SP-T</t>
+          <t>P3050ALC</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>B0H3MGC36H</t>
+          <t>B0H6C92MLT</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -4855,19 +4855,19 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>462.37</v>
+        <v>623.5</v>
       </c>
       <c r="E99" t="n">
-        <v>416.13</v>
+        <v>561.15</v>
       </c>
       <c r="F99" t="n">
-        <v>15.7</v>
+        <v>14.1</v>
       </c>
       <c r="G99" t="n">
-        <v>12.6</v>
+        <v>10.8</v>
       </c>
       <c r="H99" t="n">
-        <v>10.5</v>
+        <v>8.6</v>
       </c>
       <c r="I99" t="n">
         <v>1</v>
@@ -4879,7 +4879,7 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>política (nicho fumo / inelegibilidade) — não expor</t>
+          <t>abaixo do piso a 10% (14.1%)</t>
         </is>
       </c>
     </row>
@@ -5549,12 +5549,12 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>FORA</t>
+          <t>FORA (recomendação)</t>
         </is>
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>política (nicho fumo / inelegibilidade) — não expor</t>
+          <t>anúncio suspenso por política (caso 21652133321 encerrado com contestação negada); margem ok (17,0%), mas a promoção passa por revisão e expõe o SKU — não expor</t>
         </is>
       </c>
     </row>

</xml_diff>